<commit_message>
add xlsx sheets to analyze results
</commit_message>
<xml_diff>
--- a/Finetuning experiment/report/results_Qwen2.5-3B.xlsx
+++ b/Finetuning experiment/report/results_Qwen2.5-3B.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vnpnk\Documents\TUM\studies\semester 2\Terminology translation\terminology-translation\Finetuning experiment\report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1ABEDB16-E5A3-4756-8596-6B46279FC542}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1FF36FE6-9A78-4C07-A4F7-BC88E1089CE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="main_results" sheetId="1" r:id="rId1"/>

</xml_diff>